<commit_message>
daily official calendar refresh 2026-07-23 11:27:54 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -18,6 +18,8 @@
     <sheet name="来源监控" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="更新日志" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="口径说明" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="官方校历刷新日志" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="官方校历命中明细" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'省份日历_人数底表'!$A$1:$AG$32</definedName>
@@ -32,9 +34,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy/m/d"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy/m/d"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -97,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -105,7 +106,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -122,6 +123,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -201,7 +205,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -437,7 +440,6 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -1230,10 +1232,10 @@
           <t>北京市</t>
         </is>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -1247,10 +1249,10 @@
       <c r="G2" s="5" t="n">
         <v>0.07572383073496659</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="H2" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="I2" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -1264,10 +1266,10 @@
       <c r="L2" s="5" t="n">
         <v>0.04072398190045249</v>
       </c>
-      <c r="M2" s="3" t="n">
+      <c r="M2" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="N2" s="3" t="n">
+      <c r="N2" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O2" s="4" t="inlineStr">
@@ -1281,10 +1283,10 @@
       <c r="Q2" s="5" t="n">
         <v>0.03998788245986064</v>
       </c>
-      <c r="R2" s="3" t="n">
+      <c r="R2" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="S2" s="3" t="n">
+      <c r="S2" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T2" s="4" t="inlineStr">
@@ -1298,10 +1300,10 @@
       <c r="V2" s="5" t="n">
         <v>0.0430379746835443</v>
       </c>
-      <c r="W2" s="3" t="n">
+      <c r="W2" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="X2" s="3" t="n">
+      <c r="X2" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y2" s="4" t="inlineStr">
@@ -1315,10 +1317,10 @@
       <c r="AA2" s="5" t="n">
         <v>0.03715355805243446</v>
       </c>
-      <c r="AB2" s="3" t="n">
+      <c r="AB2" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="AC2" s="3" t="n">
+      <c r="AC2" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD2" s="4" t="inlineStr">
@@ -1347,10 +1349,10 @@
           <t>天津市</t>
         </is>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -1364,10 +1366,10 @@
       <c r="G3" s="5" t="n">
         <v>0.02524127691165553</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="H3" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="I3" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -1381,10 +1383,10 @@
       <c r="L3" s="5" t="n">
         <v>0.01844761573268361</v>
       </c>
-      <c r="M3" s="3" t="n">
+      <c r="M3" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="N3" s="3" t="n">
+      <c r="N3" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O3" s="4" t="inlineStr">
@@ -1398,10 +1400,10 @@
       <c r="Q3" s="5" t="n">
         <v>0.01423810966373826</v>
       </c>
-      <c r="R3" s="3" t="n">
+      <c r="R3" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="S3" s="3" t="n">
+      <c r="S3" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T3" s="4" t="inlineStr">
@@ -1415,10 +1417,10 @@
       <c r="V3" s="5" t="n">
         <v>0.01703992210321324</v>
       </c>
-      <c r="W3" s="3" t="n">
+      <c r="W3" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="X3" s="3" t="n">
+      <c r="X3" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y3" s="4" t="inlineStr">
@@ -1432,10 +1434,10 @@
       <c r="AA3" s="5" t="n">
         <v>0.01595505617977528</v>
       </c>
-      <c r="AB3" s="3" t="n">
+      <c r="AB3" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="AC3" s="3" t="n">
+      <c r="AC3" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD3" s="4" t="inlineStr">
@@ -1464,10 +1466,10 @@
           <t>河北省</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -1481,10 +1483,10 @@
       <c r="G4" s="5" t="n">
         <v>0.03192279138827023</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="H4" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="I4" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -1498,10 +1500,10 @@
       <c r="L4" s="5" t="n">
         <v>0.03863557257222416</v>
       </c>
-      <c r="M4" s="3" t="n">
+      <c r="M4" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="N4" s="3" t="n">
+      <c r="N4" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O4" s="4" t="inlineStr">
@@ -1515,10 +1517,10 @@
       <c r="Q4" s="5" t="n">
         <v>0.0421084519842472</v>
       </c>
-      <c r="R4" s="3" t="n">
+      <c r="R4" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="S4" s="3" t="n">
+      <c r="S4" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T4" s="4" t="inlineStr">
@@ -1532,10 +1534,10 @@
       <c r="V4" s="5" t="n">
         <v>0.04595910418695229</v>
       </c>
-      <c r="W4" s="3" t="n">
+      <c r="W4" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="X4" s="3" t="n">
+      <c r="X4" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y4" s="4" t="inlineStr">
@@ -1549,10 +1551,10 @@
       <c r="AA4" s="5" t="n">
         <v>0.04348314606741573</v>
       </c>
-      <c r="AB4" s="3" t="n">
+      <c r="AB4" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="AC4" s="3" t="n">
+      <c r="AC4" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD4" s="4" t="inlineStr">
@@ -1581,10 +1583,10 @@
           <t>山西省</t>
         </is>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -1598,10 +1600,10 @@
       <c r="G5" s="5" t="n">
         <v>0.02301410541945063</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="H5" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="I5" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -1615,10 +1617,10 @@
       <c r="L5" s="5" t="n">
         <v>0.02888966237382527</v>
       </c>
-      <c r="M5" s="3" t="n">
+      <c r="M5" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="N5" s="3" t="n">
+      <c r="N5" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O5" s="4" t="inlineStr">
@@ -1632,10 +1634,10 @@
       <c r="Q5" s="5" t="n">
         <v>0.02999091184489549</v>
       </c>
-      <c r="R5" s="3" t="n">
+      <c r="R5" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="S5" s="3" t="n">
+      <c r="S5" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T5" s="4" t="inlineStr">
@@ -1649,10 +1651,10 @@
       <c r="V5" s="5" t="n">
         <v>0.02891918208373905</v>
       </c>
-      <c r="W5" s="3" t="n">
+      <c r="W5" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="X5" s="3" t="n">
+      <c r="X5" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y5" s="4" t="inlineStr">
@@ -1666,10 +1668,10 @@
       <c r="AA5" s="5" t="n">
         <v>0.04176029962546816</v>
       </c>
-      <c r="AB5" s="3" t="n">
+      <c r="AB5" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="AC5" s="3" t="n">
+      <c r="AC5" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD5" s="4" t="inlineStr">
@@ -1698,10 +1700,10 @@
           <t>内蒙古自治区</t>
         </is>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="9" t="n">
         <v>46397</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -1715,10 +1717,10 @@
       <c r="G6" s="5" t="n">
         <v>0.0311804008908686</v>
       </c>
-      <c r="H6" s="3" t="n">
+      <c r="H6" s="9" t="n">
         <v>46397</v>
       </c>
-      <c r="I6" s="3" t="n">
+      <c r="I6" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -1732,10 +1734,10 @@
       <c r="L6" s="5" t="n">
         <v>0.02993386703793944</v>
       </c>
-      <c r="M6" s="3" t="n">
+      <c r="M6" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="N6" s="3" t="n">
+      <c r="N6" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O6" s="4" t="inlineStr">
@@ -1749,10 +1751,10 @@
       <c r="Q6" s="5" t="n">
         <v>0.02059981823689791</v>
       </c>
-      <c r="R6" s="3" t="n">
+      <c r="R6" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="S6" s="3" t="n">
+      <c r="S6" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T6" s="4" t="inlineStr">
@@ -1766,10 +1768,10 @@
       <c r="V6" s="5" t="n">
         <v>0.01645569620253165</v>
       </c>
-      <c r="W6" s="3" t="n">
+      <c r="W6" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="X6" s="3" t="n">
+      <c r="X6" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y6" s="4" t="inlineStr">
@@ -1783,10 +1785,10 @@
       <c r="AA6" s="5" t="n">
         <v>0.0200749063670412</v>
       </c>
-      <c r="AB6" s="3" t="n">
+      <c r="AB6" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="AC6" s="3" t="n">
+      <c r="AC6" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD6" s="4" t="inlineStr">
@@ -1815,10 +1817,10 @@
           <t>辽宁省</t>
         </is>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D7" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -1832,10 +1834,10 @@
       <c r="G7" s="5" t="n">
         <v>0.03563474387527839</v>
       </c>
-      <c r="H7" s="3" t="n">
+      <c r="H7" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="I7" s="3" t="n">
+      <c r="I7" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -1849,10 +1851,10 @@
       <c r="L7" s="5" t="n">
         <v>0.01844761573268361</v>
       </c>
-      <c r="M7" s="3" t="n">
+      <c r="M7" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="N7" s="3" t="n">
+      <c r="N7" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O7" s="4" t="inlineStr">
@@ -1866,10 +1868,10 @@
       <c r="Q7" s="5" t="n">
         <v>0.01908512571947895</v>
       </c>
-      <c r="R7" s="3" t="n">
+      <c r="R7" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="S7" s="3" t="n">
+      <c r="S7" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T7" s="4" t="inlineStr">
@@ -1883,10 +1885,10 @@
       <c r="V7" s="5" t="n">
         <v>0.02833495618305745</v>
       </c>
-      <c r="W7" s="3" t="n">
+      <c r="W7" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="X7" s="3" t="n">
+      <c r="X7" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y7" s="4" t="inlineStr">
@@ -1900,10 +1902,10 @@
       <c r="AA7" s="5" t="n">
         <v>0.02359550561797753</v>
       </c>
-      <c r="AB7" s="3" t="n">
+      <c r="AB7" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="AC7" s="3" t="n">
+      <c r="AC7" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD7" s="4" t="inlineStr">
@@ -1932,10 +1934,10 @@
           <t>吉林省</t>
         </is>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="9" t="n">
         <v>46397</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -1949,10 +1951,10 @@
       <c r="G8" s="5" t="n">
         <v>0.008908685968819599</v>
       </c>
-      <c r="H8" s="3" t="n">
+      <c r="H8" s="9" t="n">
         <v>46397</v>
       </c>
-      <c r="I8" s="3" t="n">
+      <c r="I8" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1966,10 +1968,10 @@
       <c r="L8" s="5" t="n">
         <v>0.01044204664114166</v>
       </c>
-      <c r="M8" s="3" t="n">
+      <c r="M8" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="N8" s="3" t="n">
+      <c r="N8" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O8" s="4" t="inlineStr">
@@ -1983,10 +1985,10 @@
       <c r="Q8" s="5" t="n">
         <v>0.006058770069675856</v>
       </c>
-      <c r="R8" s="3" t="n">
+      <c r="R8" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="S8" s="3" t="n">
+      <c r="S8" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T8" s="4" t="inlineStr">
@@ -2000,10 +2002,10 @@
       <c r="V8" s="5" t="n">
         <v>0.01392405063291139</v>
       </c>
-      <c r="W8" s="3" t="n">
+      <c r="W8" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="X8" s="3" t="n">
+      <c r="X8" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y8" s="4" t="inlineStr">
@@ -2017,10 +2019,10 @@
       <c r="AA8" s="5" t="n">
         <v>0.01269662921348315</v>
       </c>
-      <c r="AB8" s="3" t="n">
+      <c r="AB8" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="AC8" s="3" t="n">
+      <c r="AC8" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD8" s="4" t="inlineStr">
@@ -2049,10 +2051,10 @@
           <t>黑龙江省</t>
         </is>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C9" s="9" t="n">
         <v>46397</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D9" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -2066,10 +2068,10 @@
       <c r="G9" s="5" t="n">
         <v>0.01410541945063103</v>
       </c>
-      <c r="H9" s="3" t="n">
+      <c r="H9" s="9" t="n">
         <v>46397</v>
       </c>
-      <c r="I9" s="3" t="n">
+      <c r="I9" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -2083,10 +2085,10 @@
       <c r="L9" s="5" t="n">
         <v>0.009745910198398886</v>
       </c>
-      <c r="M9" s="3" t="n">
+      <c r="M9" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="N9" s="3" t="n">
+      <c r="N9" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O9" s="4" t="inlineStr">
@@ -2100,10 +2102,10 @@
       <c r="Q9" s="5" t="n">
         <v>0.0127234171463193</v>
       </c>
-      <c r="R9" s="3" t="n">
+      <c r="R9" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="S9" s="3" t="n">
+      <c r="S9" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T9" s="4" t="inlineStr">
@@ -2117,10 +2119,10 @@
       <c r="V9" s="5" t="n">
         <v>0.01635832521908471</v>
       </c>
-      <c r="W9" s="3" t="n">
+      <c r="W9" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="X9" s="3" t="n">
+      <c r="X9" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y9" s="4" t="inlineStr">
@@ -2134,10 +2136,10 @@
       <c r="AA9" s="5" t="n">
         <v>0.01951310861423221</v>
       </c>
-      <c r="AB9" s="3" t="n">
+      <c r="AB9" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="AC9" s="3" t="n">
+      <c r="AC9" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD9" s="4" t="inlineStr">
@@ -2166,10 +2168,10 @@
           <t>上海市</t>
         </is>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -2183,10 +2185,10 @@
       <c r="G10" s="5" t="n">
         <v>0.0289532293986637</v>
       </c>
-      <c r="H10" s="3" t="n">
+      <c r="H10" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="I10" s="3" t="n">
+      <c r="I10" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -2200,10 +2202,10 @@
       <c r="L10" s="5" t="n">
         <v>0.02888966237382527</v>
       </c>
-      <c r="M10" s="3" t="n">
+      <c r="M10" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="N10" s="3" t="n">
+      <c r="N10" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O10" s="4" t="inlineStr">
@@ -2217,10 +2219,10 @@
       <c r="Q10" s="5" t="n">
         <v>0.0293850348379279</v>
       </c>
-      <c r="R10" s="3" t="n">
+      <c r="R10" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="S10" s="3" t="n">
+      <c r="S10" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T10" s="4" t="inlineStr">
@@ -2234,10 +2236,10 @@
       <c r="V10" s="5" t="n">
         <v>0.01509250243427459</v>
       </c>
-      <c r="W10" s="3" t="n">
+      <c r="W10" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="X10" s="3" t="n">
+      <c r="X10" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y10" s="4" t="inlineStr">
@@ -2251,10 +2253,10 @@
       <c r="AA10" s="5" t="n">
         <v>0.0149812734082397</v>
       </c>
-      <c r="AB10" s="3" t="n">
+      <c r="AB10" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="AC10" s="3" t="n">
+      <c r="AC10" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD10" s="4" t="inlineStr">
@@ -2283,10 +2285,10 @@
           <t>江苏省</t>
         </is>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="C11" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D11" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -2300,10 +2302,10 @@
       <c r="G11" s="5" t="n">
         <v>0.08834446919079436</v>
       </c>
-      <c r="H11" s="3" t="n">
+      <c r="H11" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="I11" s="3" t="n">
+      <c r="I11" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -2317,10 +2319,10 @@
       <c r="L11" s="5" t="n">
         <v>0.08318830490776193</v>
       </c>
-      <c r="M11" s="3" t="n">
+      <c r="M11" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="N11" s="3" t="n">
+      <c r="N11" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O11" s="4" t="inlineStr">
@@ -2334,10 +2336,10 @@
       <c r="Q11" s="5" t="n">
         <v>0.09179036655558921</v>
       </c>
-      <c r="R11" s="3" t="n">
+      <c r="R11" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="S11" s="3" t="n">
+      <c r="S11" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T11" s="4" t="inlineStr">
@@ -2351,10 +2353,10 @@
       <c r="V11" s="5" t="n">
         <v>0.1024342745861733</v>
       </c>
-      <c r="W11" s="3" t="n">
+      <c r="W11" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="X11" s="3" t="n">
+      <c r="X11" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y11" s="4" t="inlineStr">
@@ -2368,10 +2370,10 @@
       <c r="AA11" s="5" t="n">
         <v>0.09157303370786517</v>
       </c>
-      <c r="AB11" s="3" t="n">
+      <c r="AB11" s="9" t="n">
         <v>46419</v>
       </c>
-      <c r="AC11" s="3" t="n">
+      <c r="AC11" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD11" s="4" t="inlineStr">
@@ -2400,10 +2402,10 @@
           <t>浙江省</t>
         </is>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="C12" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D12" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -2417,10 +2419,10 @@
       <c r="G12" s="5" t="n">
         <v>0.09428359317000742</v>
       </c>
-      <c r="H12" s="3" t="n">
+      <c r="H12" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="I12" s="3" t="n">
+      <c r="I12" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -2434,10 +2436,10 @@
       <c r="L12" s="5" t="n">
         <v>0.07970762269404803</v>
       </c>
-      <c r="M12" s="3" t="n">
+      <c r="M12" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="N12" s="3" t="n">
+      <c r="N12" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O12" s="4" t="inlineStr">
@@ -2451,10 +2453,10 @@
       <c r="Q12" s="5" t="n">
         <v>0.06967585580127234</v>
       </c>
-      <c r="R12" s="3" t="n">
+      <c r="R12" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="S12" s="3" t="n">
+      <c r="S12" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T12" s="4" t="inlineStr">
@@ -2468,10 +2470,10 @@
       <c r="V12" s="5" t="n">
         <v>0.08481012658227848</v>
       </c>
-      <c r="W12" s="3" t="n">
+      <c r="W12" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="X12" s="3" t="n">
+      <c r="X12" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y12" s="4" t="inlineStr">
@@ -2485,10 +2487,10 @@
       <c r="AA12" s="5" t="n">
         <v>0.06947565543071162</v>
       </c>
-      <c r="AB12" s="3" t="n">
+      <c r="AB12" s="9" t="n">
         <v>46419</v>
       </c>
-      <c r="AC12" s="3" t="n">
+      <c r="AC12" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD12" s="4" t="inlineStr">
@@ -2517,10 +2519,10 @@
           <t>安徽省</t>
         </is>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="C13" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D13" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -2534,10 +2536,10 @@
       <c r="G13" s="5" t="n">
         <v>0.02746844840386043</v>
       </c>
-      <c r="H13" s="3" t="n">
+      <c r="H13" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="I13" s="3" t="n">
+      <c r="I13" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -2551,10 +2553,10 @@
       <c r="L13" s="5" t="n">
         <v>0.04942568743473721</v>
       </c>
-      <c r="M13" s="3" t="n">
+      <c r="M13" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="N13" s="3" t="n">
+      <c r="N13" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O13" s="4" t="inlineStr">
@@ -2568,10 +2570,10 @@
       <c r="Q13" s="5" t="n">
         <v>0.04392608300514995</v>
       </c>
-      <c r="R13" s="3" t="n">
+      <c r="R13" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="S13" s="3" t="n">
+      <c r="S13" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
@@ -2585,10 +2587,10 @@
       <c r="V13" s="5" t="n">
         <v>0.05170399221032133</v>
       </c>
-      <c r="W13" s="3" t="n">
+      <c r="W13" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="X13" s="3" t="n">
+      <c r="X13" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y13" s="4" t="inlineStr">
@@ -2602,10 +2604,10 @@
       <c r="AA13" s="5" t="n">
         <v>0.04363295880149812</v>
       </c>
-      <c r="AB13" s="3" t="n">
+      <c r="AB13" s="9" t="n">
         <v>46419</v>
       </c>
-      <c r="AC13" s="3" t="n">
+      <c r="AC13" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD13" s="4" t="inlineStr">
@@ -2634,10 +2636,10 @@
           <t>福建省</t>
         </is>
       </c>
-      <c r="C14" s="3" t="n">
+      <c r="C14" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -2651,10 +2653,10 @@
       <c r="G14" s="5" t="n">
         <v>0.03192279138827023</v>
       </c>
-      <c r="H14" s="3" t="n">
+      <c r="H14" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="I14" s="3" t="n">
+      <c r="I14" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -2668,10 +2670,10 @@
       <c r="L14" s="5" t="n">
         <v>0.03759136790810999</v>
       </c>
-      <c r="M14" s="3" t="n">
+      <c r="M14" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="N14" s="3" t="n">
+      <c r="N14" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O14" s="4" t="inlineStr">
@@ -2685,10 +2687,10 @@
       <c r="Q14" s="5" t="n">
         <v>0.04725840654347167</v>
       </c>
-      <c r="R14" s="3" t="n">
+      <c r="R14" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="S14" s="3" t="n">
+      <c r="S14" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T14" s="4" t="inlineStr">
@@ -2702,10 +2704,10 @@
       <c r="V14" s="5" t="n">
         <v>0.02814021421616358</v>
       </c>
-      <c r="W14" s="3" t="n">
+      <c r="W14" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="X14" s="3" t="n">
+      <c r="X14" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y14" s="4" t="inlineStr">
@@ -2719,10 +2721,10 @@
       <c r="AA14" s="5" t="n">
         <v>0.02865168539325843</v>
       </c>
-      <c r="AB14" s="3" t="n">
+      <c r="AB14" s="9" t="n">
         <v>46419</v>
       </c>
-      <c r="AC14" s="3" t="n">
+      <c r="AC14" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD14" s="4" t="inlineStr">
@@ -2751,10 +2753,10 @@
           <t>江西省</t>
         </is>
       </c>
-      <c r="C15" s="3" t="n">
+      <c r="C15" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -2768,10 +2770,10 @@
       <c r="G15" s="5" t="n">
         <v>0.02152932442464736</v>
       </c>
-      <c r="H15" s="3" t="n">
+      <c r="H15" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="I15" s="3" t="n">
+      <c r="I15" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -2785,10 +2787,10 @@
       <c r="L15" s="5" t="n">
         <v>0.02540898016011138</v>
       </c>
-      <c r="M15" s="3" t="n">
+      <c r="M15" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="N15" s="3" t="n">
+      <c r="N15" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O15" s="4" t="inlineStr">
@@ -2802,10 +2804,10 @@
       <c r="Q15" s="5" t="n">
         <v>0.0293850348379279</v>
       </c>
-      <c r="R15" s="3" t="n">
+      <c r="R15" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="S15" s="3" t="n">
+      <c r="S15" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
@@ -2819,10 +2821,10 @@
       <c r="V15" s="5" t="n">
         <v>0.02814021421616358</v>
       </c>
-      <c r="W15" s="3" t="n">
+      <c r="W15" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="X15" s="3" t="n">
+      <c r="X15" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y15" s="4" t="inlineStr">
@@ -2836,10 +2838,10 @@
       <c r="AA15" s="5" t="n">
         <v>0.02606741573033708</v>
       </c>
-      <c r="AB15" s="3" t="n">
+      <c r="AB15" s="9" t="n">
         <v>46419</v>
       </c>
-      <c r="AC15" s="3" t="n">
+      <c r="AC15" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD15" s="4" t="inlineStr">
@@ -2868,10 +2870,10 @@
           <t>山东省</t>
         </is>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="C16" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -2885,10 +2887,10 @@
       <c r="G16" s="5" t="n">
         <v>0.06087602078693393</v>
       </c>
-      <c r="H16" s="3" t="n">
+      <c r="H16" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="I16" s="3" t="n">
+      <c r="I16" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -2902,10 +2904,10 @@
       <c r="L16" s="5" t="n">
         <v>0.06056387051862165</v>
       </c>
-      <c r="M16" s="3" t="n">
+      <c r="M16" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="N16" s="3" t="n">
+      <c r="N16" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O16" s="4" t="inlineStr">
@@ -2919,10 +2921,10 @@
       <c r="Q16" s="5" t="n">
         <v>0.0590730081793396</v>
       </c>
-      <c r="R16" s="3" t="n">
+      <c r="R16" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="S16" s="3" t="n">
+      <c r="S16" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T16" s="4" t="inlineStr">
@@ -2936,10 +2938,10 @@
       <c r="V16" s="5" t="n">
         <v>0.06893865628042843</v>
       </c>
-      <c r="W16" s="3" t="n">
+      <c r="W16" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="X16" s="3" t="n">
+      <c r="X16" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y16" s="4" t="inlineStr">
@@ -2953,10 +2955,10 @@
       <c r="AA16" s="5" t="n">
         <v>0.08033707865168539</v>
       </c>
-      <c r="AB16" s="3" t="n">
+      <c r="AB16" s="9" t="n">
         <v>46419</v>
       </c>
-      <c r="AC16" s="3" t="n">
+      <c r="AC16" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD16" s="4" t="inlineStr">
@@ -2985,10 +2987,10 @@
           <t>河南省</t>
         </is>
       </c>
-      <c r="C17" s="3" t="n">
+      <c r="C17" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D17" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -3002,10 +3004,10 @@
       <c r="G17" s="5" t="n">
         <v>0.03711952487008166</v>
       </c>
-      <c r="H17" s="3" t="n">
+      <c r="H17" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="I17" s="3" t="n">
+      <c r="I17" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -3019,10 +3021,10 @@
       <c r="L17" s="5" t="n">
         <v>0.03828750435085277</v>
       </c>
-      <c r="M17" s="3" t="n">
+      <c r="M17" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="N17" s="3" t="n">
+      <c r="N17" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O17" s="4" t="inlineStr">
@@ -3036,10 +3038,10 @@
       <c r="Q17" s="5" t="n">
         <v>0.0418055134807634</v>
       </c>
-      <c r="R17" s="3" t="n">
+      <c r="R17" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="S17" s="3" t="n">
+      <c r="S17" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
@@ -3053,10 +3055,10 @@
       <c r="V17" s="5" t="n">
         <v>0.05141187925998052</v>
       </c>
-      <c r="W17" s="3" t="n">
+      <c r="W17" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="X17" s="3" t="n">
+      <c r="X17" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y17" s="4" t="inlineStr">
@@ -3070,10 +3072,10 @@
       <c r="AA17" s="5" t="n">
         <v>0.05910112359550562</v>
       </c>
-      <c r="AB17" s="3" t="n">
+      <c r="AB17" s="9" t="n">
         <v>46419</v>
       </c>
-      <c r="AC17" s="3" t="n">
+      <c r="AC17" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD17" s="4" t="inlineStr">
@@ -3102,10 +3104,10 @@
           <t>湖北省</t>
         </is>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="C18" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D18" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -3119,10 +3121,10 @@
       <c r="G18" s="5" t="n">
         <v>0.03266518188567186</v>
       </c>
-      <c r="H18" s="3" t="n">
+      <c r="H18" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="I18" s="3" t="n">
+      <c r="I18" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -3136,10 +3138,10 @@
       <c r="L18" s="5" t="n">
         <v>0.03759136790810999</v>
       </c>
-      <c r="M18" s="3" t="n">
+      <c r="M18" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="N18" s="3" t="n">
+      <c r="N18" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O18" s="4" t="inlineStr">
@@ -3153,10 +3155,10 @@
       <c r="Q18" s="5" t="n">
         <v>0.02968797334141169</v>
       </c>
-      <c r="R18" s="3" t="n">
+      <c r="R18" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="S18" s="3" t="n">
+      <c r="S18" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T18" s="4" t="inlineStr">
@@ -3170,10 +3172,10 @@
       <c r="V18" s="5" t="n">
         <v>0.04167478091528724</v>
       </c>
-      <c r="W18" s="3" t="n">
+      <c r="W18" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="X18" s="3" t="n">
+      <c r="X18" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y18" s="4" t="inlineStr">
@@ -3187,10 +3189,10 @@
       <c r="AA18" s="5" t="n">
         <v>0.03928838951310861</v>
       </c>
-      <c r="AB18" s="3" t="n">
+      <c r="AB18" s="9" t="n">
         <v>46419</v>
       </c>
-      <c r="AC18" s="3" t="n">
+      <c r="AC18" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD18" s="4" t="inlineStr">
@@ -3219,10 +3221,10 @@
           <t>湖南省</t>
         </is>
       </c>
-      <c r="C19" s="3" t="n">
+      <c r="C19" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="D19" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -3236,10 +3238,10 @@
       <c r="G19" s="5" t="n">
         <v>0.04157386785449146</v>
       </c>
-      <c r="H19" s="3" t="n">
+      <c r="H19" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="I19" s="3" t="n">
+      <c r="I19" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -3253,10 +3255,10 @@
       <c r="L19" s="5" t="n">
         <v>0.0435085276714236</v>
       </c>
-      <c r="M19" s="3" t="n">
+      <c r="M19" s="9" t="n">
         <v>46412</v>
       </c>
-      <c r="N19" s="3" t="n">
+      <c r="N19" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O19" s="4" t="inlineStr">
@@ -3270,10 +3272,10 @@
       <c r="Q19" s="5" t="n">
         <v>0.05089366858527719</v>
       </c>
-      <c r="R19" s="3" t="n">
+      <c r="R19" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="S19" s="3" t="n">
+      <c r="S19" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
@@ -3287,10 +3289,10 @@
       <c r="V19" s="5" t="n">
         <v>0.04050632911392405</v>
       </c>
-      <c r="W19" s="3" t="n">
+      <c r="W19" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="X19" s="3" t="n">
+      <c r="X19" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y19" s="4" t="inlineStr">
@@ -3304,10 +3306,10 @@
       <c r="AA19" s="5" t="n">
         <v>0.04213483146067416</v>
       </c>
-      <c r="AB19" s="3" t="n">
+      <c r="AB19" s="9" t="n">
         <v>46419</v>
       </c>
-      <c r="AC19" s="3" t="n">
+      <c r="AC19" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD19" s="4" t="inlineStr">
@@ -3336,10 +3338,10 @@
           <t>广东省</t>
         </is>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="C20" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D20" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -3353,10 +3355,10 @@
       <c r="G20" s="5" t="n">
         <v>0.1061618411284336</v>
       </c>
-      <c r="H20" s="3" t="n">
+      <c r="H20" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="I20" s="3" t="n">
+      <c r="I20" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -3370,10 +3372,10 @@
       <c r="L20" s="5" t="n">
         <v>0.106508875739645</v>
       </c>
-      <c r="M20" s="3" t="n">
+      <c r="M20" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="N20" s="3" t="n">
+      <c r="N20" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O20" s="4" t="inlineStr">
@@ -3387,10 +3389,10 @@
       <c r="Q20" s="5" t="n">
         <v>0.1145107543168737</v>
       </c>
-      <c r="R20" s="3" t="n">
+      <c r="R20" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="S20" s="3" t="n">
+      <c r="S20" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T20" s="4" t="inlineStr">
@@ -3404,10 +3406,10 @@
       <c r="V20" s="5" t="n">
         <v>0.07448880233690361</v>
       </c>
-      <c r="W20" s="3" t="n">
+      <c r="W20" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="X20" s="3" t="n">
+      <c r="X20" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y20" s="4" t="inlineStr">
@@ -3421,10 +3423,10 @@
       <c r="AA20" s="5" t="n">
         <v>0.09224719101123595</v>
       </c>
-      <c r="AB20" s="3" t="n">
+      <c r="AB20" s="9" t="n">
         <v>46419</v>
       </c>
-      <c r="AC20" s="3" t="n">
+      <c r="AC20" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD20" s="4" t="inlineStr">
@@ -3453,10 +3455,10 @@
           <t>广西壮族自治区</t>
         </is>
       </c>
-      <c r="C21" s="3" t="n">
+      <c r="C21" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D21" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -3470,10 +3472,10 @@
       <c r="G21" s="5" t="n">
         <v>0.02301410541945063</v>
       </c>
-      <c r="H21" s="3" t="n">
+      <c r="H21" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="I21" s="3" t="n">
+      <c r="I21" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -3487,10 +3489,10 @@
       <c r="L21" s="5" t="n">
         <v>0.02123216150365472</v>
       </c>
-      <c r="M21" s="3" t="n">
+      <c r="M21" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="N21" s="3" t="n">
+      <c r="N21" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O21" s="4" t="inlineStr">
@@ -3504,10 +3506,10 @@
       <c r="Q21" s="5" t="n">
         <v>0.01969100272644653</v>
       </c>
-      <c r="R21" s="3" t="n">
+      <c r="R21" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="S21" s="3" t="n">
+      <c r="S21" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
@@ -3521,10 +3523,10 @@
       <c r="V21" s="5" t="n">
         <v>0.01996105160662123</v>
       </c>
-      <c r="W21" s="3" t="n">
+      <c r="W21" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="X21" s="3" t="n">
+      <c r="X21" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y21" s="4" t="inlineStr">
@@ -3538,10 +3540,10 @@
       <c r="AA21" s="5" t="n">
         <v>0.01816479400749064</v>
       </c>
-      <c r="AB21" s="3" t="n">
+      <c r="AB21" s="9" t="n">
         <v>46419</v>
       </c>
-      <c r="AC21" s="3" t="n">
+      <c r="AC21" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD21" s="4" t="inlineStr">
@@ -3570,10 +3572,10 @@
           <t>海南省</t>
         </is>
       </c>
-      <c r="C22" s="3" t="n">
+      <c r="C22" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="D22" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -3587,10 +3589,10 @@
       <c r="G22" s="5" t="n">
         <v>0.003711952487008166</v>
       </c>
-      <c r="H22" s="3" t="n">
+      <c r="H22" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="I22" s="3" t="n">
+      <c r="I22" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -3604,10 +3606,10 @@
       <c r="L22" s="5" t="n">
         <v>0.008005569091541943</v>
       </c>
-      <c r="M22" s="3" t="n">
+      <c r="M22" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="N22" s="3" t="n">
+      <c r="N22" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O22" s="4" t="inlineStr">
@@ -3621,10 +3623,10 @@
       <c r="Q22" s="5" t="n">
         <v>0.006361708573159649</v>
       </c>
-      <c r="R22" s="3" t="n">
+      <c r="R22" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="S22" s="3" t="n">
+      <c r="S22" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T22" s="4" t="inlineStr">
@@ -3638,10 +3640,10 @@
       <c r="V22" s="5" t="n">
         <v>0.006037000973709835</v>
       </c>
-      <c r="W22" s="3" t="n">
+      <c r="W22" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="X22" s="3" t="n">
+      <c r="X22" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y22" s="4" t="inlineStr">
@@ -3655,10 +3657,10 @@
       <c r="AA22" s="5" t="n">
         <v>0.005917602996254681</v>
       </c>
-      <c r="AB22" s="3" t="n">
+      <c r="AB22" s="9" t="n">
         <v>46419</v>
       </c>
-      <c r="AC22" s="3" t="n">
+      <c r="AC22" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD22" s="4" t="inlineStr">
@@ -3687,10 +3689,10 @@
           <t>重庆市</t>
         </is>
       </c>
-      <c r="C23" s="3" t="n">
+      <c r="C23" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D23" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -3704,10 +3706,10 @@
       <c r="G23" s="5" t="n">
         <v>0.01930215293244246</v>
       </c>
-      <c r="H23" s="3" t="n">
+      <c r="H23" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="I23" s="3" t="n">
+      <c r="I23" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -3721,10 +3723,10 @@
       <c r="L23" s="5" t="n">
         <v>0.01914375217542639</v>
       </c>
-      <c r="M23" s="3" t="n">
+      <c r="M23" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="N23" s="3" t="n">
+      <c r="N23" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O23" s="4" t="inlineStr">
@@ -3738,10 +3740,10 @@
       <c r="Q23" s="5" t="n">
         <v>0.01726749469857619</v>
       </c>
-      <c r="R23" s="3" t="n">
+      <c r="R23" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="S23" s="3" t="n">
+      <c r="S23" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
@@ -3755,10 +3757,10 @@
       <c r="V23" s="5" t="n">
         <v>0.02385589094449854</v>
       </c>
-      <c r="W23" s="3" t="n">
+      <c r="W23" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="X23" s="3" t="n">
+      <c r="X23" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y23" s="4" t="inlineStr">
@@ -3772,10 +3774,10 @@
       <c r="AA23" s="5" t="n">
         <v>0.0200749063670412</v>
       </c>
-      <c r="AB23" s="3" t="n">
+      <c r="AB23" s="9" t="n">
         <v>46419</v>
       </c>
-      <c r="AC23" s="3" t="n">
+      <c r="AC23" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD23" s="4" t="inlineStr">
@@ -3804,10 +3806,10 @@
           <t>四川省</t>
         </is>
       </c>
-      <c r="C24" s="3" t="n">
+      <c r="C24" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="D24" s="3" t="n">
+      <c r="D24" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -3821,10 +3823,10 @@
       <c r="G24" s="5" t="n">
         <v>0.04899777282850779</v>
       </c>
-      <c r="H24" s="3" t="n">
+      <c r="H24" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="I24" s="3" t="n">
+      <c r="I24" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -3838,10 +3840,10 @@
       <c r="L24" s="5" t="n">
         <v>0.04872955099199443</v>
       </c>
-      <c r="M24" s="3" t="n">
+      <c r="M24" s="9" t="n">
         <v>46417</v>
       </c>
-      <c r="N24" s="3" t="n">
+      <c r="N24" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O24" s="4" t="inlineStr">
@@ -3855,10 +3857,10 @@
       <c r="Q24" s="5" t="n">
         <v>0.04877309906089064</v>
       </c>
-      <c r="R24" s="3" t="n">
+      <c r="R24" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="S24" s="3" t="n">
+      <c r="S24" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T24" s="4" t="inlineStr">
@@ -3872,10 +3874,10 @@
       <c r="V24" s="5" t="n">
         <v>0.05219084712755599</v>
       </c>
-      <c r="W24" s="3" t="n">
+      <c r="W24" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="X24" s="3" t="n">
+      <c r="X24" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y24" s="4" t="inlineStr">
@@ -3889,10 +3891,10 @@
       <c r="AA24" s="5" t="n">
         <v>0.04258426966292135</v>
       </c>
-      <c r="AB24" s="3" t="n">
+      <c r="AB24" s="9" t="n">
         <v>46419</v>
       </c>
-      <c r="AC24" s="3" t="n">
+      <c r="AC24" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD24" s="4" t="inlineStr">
@@ -3921,10 +3923,10 @@
           <t>贵州省</t>
         </is>
       </c>
-      <c r="C25" s="3" t="n">
+      <c r="C25" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="D25" s="3" t="n">
+      <c r="D25" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -3938,10 +3940,10 @@
       <c r="G25" s="5" t="n">
         <v>0.0155902004454343</v>
       </c>
-      <c r="H25" s="3" t="n">
+      <c r="H25" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="I25" s="3" t="n">
+      <c r="I25" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -3955,10 +3957,10 @@
       <c r="L25" s="5" t="n">
         <v>0.01357466063348416</v>
       </c>
-      <c r="M25" s="3" t="n">
+      <c r="M25" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="N25" s="3" t="n">
+      <c r="N25" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O25" s="4" t="inlineStr">
@@ -3972,10 +3974,10 @@
       <c r="Q25" s="5" t="n">
         <v>0.01757043320205998</v>
       </c>
-      <c r="R25" s="3" t="n">
+      <c r="R25" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="S25" s="3" t="n">
+      <c r="S25" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
@@ -3989,10 +3991,10 @@
       <c r="V25" s="5" t="n">
         <v>0.0127555988315482</v>
       </c>
-      <c r="W25" s="3" t="n">
+      <c r="W25" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="X25" s="3" t="n">
+      <c r="X25" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y25" s="4" t="inlineStr">
@@ -4006,10 +4008,10 @@
       <c r="AA25" s="5" t="n">
         <v>0.01453183520599251</v>
       </c>
-      <c r="AB25" s="3" t="n">
+      <c r="AB25" s="9" t="n">
         <v>46419</v>
       </c>
-      <c r="AC25" s="3" t="n">
+      <c r="AC25" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD25" s="4" t="inlineStr">
@@ -4038,10 +4040,10 @@
           <t>云南省</t>
         </is>
       </c>
-      <c r="C26" s="3" t="n">
+      <c r="C26" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="D26" s="3" t="n">
+      <c r="D26" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -4055,10 +4057,10 @@
       <c r="G26" s="5" t="n">
         <v>0.009651076466221232</v>
       </c>
-      <c r="H26" s="3" t="n">
+      <c r="H26" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="I26" s="3" t="n">
+      <c r="I26" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -4072,10 +4074,10 @@
       <c r="L26" s="5" t="n">
         <v>0.01740341106856944</v>
       </c>
-      <c r="M26" s="3" t="n">
+      <c r="M26" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="N26" s="3" t="n">
+      <c r="N26" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O26" s="4" t="inlineStr">
@@ -4089,10 +4091,10 @@
       <c r="Q26" s="5" t="n">
         <v>0.01817631020902757</v>
       </c>
-      <c r="R26" s="3" t="n">
+      <c r="R26" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="S26" s="3" t="n">
+      <c r="S26" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T26" s="4" t="inlineStr">
@@ -4106,10 +4108,10 @@
       <c r="V26" s="5" t="n">
         <v>0.01655306718597858</v>
       </c>
-      <c r="W26" s="3" t="n">
+      <c r="W26" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="X26" s="3" t="n">
+      <c r="X26" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y26" s="4" t="inlineStr">
@@ -4123,10 +4125,10 @@
       <c r="AA26" s="5" t="n">
         <v>0.01535580524344569</v>
       </c>
-      <c r="AB26" s="3" t="n">
+      <c r="AB26" s="9" t="n">
         <v>46419</v>
       </c>
-      <c r="AC26" s="3" t="n">
+      <c r="AC26" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD26" s="4" t="inlineStr">
@@ -4155,10 +4157,10 @@
           <t>西藏自治区</t>
         </is>
       </c>
-      <c r="C27" s="3" t="n">
+      <c r="C27" s="9" t="n">
         <v>46397</v>
       </c>
-      <c r="D27" s="3" t="n">
+      <c r="D27" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -4172,10 +4174,10 @@
       <c r="G27" s="5" t="n">
         <v>0.0007423904974016332</v>
       </c>
-      <c r="H27" s="3" t="n">
+      <c r="H27" s="9" t="n">
         <v>46397</v>
       </c>
-      <c r="I27" s="3" t="n">
+      <c r="I27" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -4189,10 +4191,10 @@
       <c r="L27" s="5" t="n">
         <v>0.001044204664114166</v>
       </c>
-      <c r="M27" s="3" t="n">
+      <c r="M27" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="N27" s="3" t="n">
+      <c r="N27" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O27" s="4" t="inlineStr">
@@ -4206,10 +4208,10 @@
       <c r="Q27" s="5" t="n">
         <v>0.001514692517418964</v>
       </c>
-      <c r="R27" s="3" t="n">
+      <c r="R27" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="S27" s="3" t="n">
+      <c r="S27" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
@@ -4223,10 +4225,10 @@
       <c r="V27" s="5" t="n">
         <v>0.0002921129503407984</v>
       </c>
-      <c r="W27" s="3" t="n">
+      <c r="W27" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="X27" s="3" t="n">
+      <c r="X27" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y27" s="4" t="inlineStr">
@@ -4240,10 +4242,10 @@
       <c r="AA27" s="5" t="n">
         <v>0.0005617977528089888</v>
       </c>
-      <c r="AB27" s="3" t="n">
+      <c r="AB27" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="AC27" s="3" t="n">
+      <c r="AC27" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD27" s="4" t="inlineStr">
@@ -4272,10 +4274,10 @@
           <t>陕西省</t>
         </is>
       </c>
-      <c r="C28" s="3" t="n">
+      <c r="C28" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="D28" s="3" t="n">
+      <c r="D28" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -4289,10 +4291,10 @@
       <c r="G28" s="5" t="n">
         <v>0.02969561989606533</v>
       </c>
-      <c r="H28" s="3" t="n">
+      <c r="H28" s="9" t="n">
         <v>46410</v>
       </c>
-      <c r="I28" s="3" t="n">
+      <c r="I28" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -4306,10 +4308,10 @@
       <c r="L28" s="5" t="n">
         <v>0.03828750435085277</v>
       </c>
-      <c r="M28" s="3" t="n">
+      <c r="M28" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="N28" s="3" t="n">
+      <c r="N28" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O28" s="4" t="inlineStr">
@@ -4323,10 +4325,10 @@
       <c r="Q28" s="5" t="n">
         <v>0.03453498939715238</v>
       </c>
-      <c r="R28" s="3" t="n">
+      <c r="R28" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="S28" s="3" t="n">
+      <c r="S28" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T28" s="4" t="inlineStr">
@@ -4340,10 +4342,10 @@
       <c r="V28" s="5" t="n">
         <v>0.02658227848101266</v>
       </c>
-      <c r="W28" s="3" t="n">
+      <c r="W28" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="X28" s="3" t="n">
+      <c r="X28" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y28" s="4" t="inlineStr">
@@ -4357,10 +4359,10 @@
       <c r="AA28" s="5" t="n">
         <v>0.03273408239700375</v>
       </c>
-      <c r="AB28" s="3" t="n">
+      <c r="AB28" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="AC28" s="3" t="n">
+      <c r="AC28" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD28" s="4" t="inlineStr">
@@ -4389,10 +4391,10 @@
           <t>甘肃省</t>
         </is>
       </c>
-      <c r="C29" s="3" t="n">
+      <c r="C29" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="D29" s="3" t="n">
+      <c r="D29" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -4406,10 +4408,10 @@
       <c r="G29" s="5" t="n">
         <v>0.01262063845582777</v>
       </c>
-      <c r="H29" s="3" t="n">
+      <c r="H29" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="I29" s="3" t="n">
+      <c r="I29" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -4423,10 +4425,10 @@
       <c r="L29" s="5" t="n">
         <v>0.01392272885485555</v>
       </c>
-      <c r="M29" s="3" t="n">
+      <c r="M29" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="N29" s="3" t="n">
+      <c r="N29" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O29" s="4" t="inlineStr">
@@ -4440,10 +4442,10 @@
       <c r="Q29" s="5" t="n">
         <v>0.01484398667070585</v>
       </c>
-      <c r="R29" s="3" t="n">
+      <c r="R29" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="S29" s="3" t="n">
+      <c r="S29" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
@@ -4457,10 +4459,10 @@
       <c r="V29" s="5" t="n">
         <v>0.01548198636806232</v>
       </c>
-      <c r="W29" s="3" t="n">
+      <c r="W29" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="X29" s="3" t="n">
+      <c r="X29" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y29" s="4" t="inlineStr">
@@ -4474,10 +4476,10 @@
       <c r="AA29" s="5" t="n">
         <v>0.01730337078651685</v>
       </c>
-      <c r="AB29" s="3" t="n">
+      <c r="AB29" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="AC29" s="3" t="n">
+      <c r="AC29" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD29" s="4" t="inlineStr">
@@ -4506,10 +4508,10 @@
           <t>青海省</t>
         </is>
       </c>
-      <c r="C30" s="3" t="n">
+      <c r="C30" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="D30" s="3" t="n">
+      <c r="D30" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -4523,10 +4525,10 @@
       <c r="G30" s="5" t="n">
         <v>0.003711952487008166</v>
       </c>
-      <c r="H30" s="3" t="n">
+      <c r="H30" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="I30" s="3" t="n">
+      <c r="I30" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -4540,10 +4542,10 @@
       <c r="L30" s="5" t="n">
         <v>0.002436477549599721</v>
       </c>
-      <c r="M30" s="3" t="n">
+      <c r="M30" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="N30" s="3" t="n">
+      <c r="N30" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O30" s="4" t="inlineStr">
@@ -4557,10 +4559,10 @@
       <c r="Q30" s="5" t="n">
         <v>0.005755831566192063</v>
       </c>
-      <c r="R30" s="3" t="n">
+      <c r="R30" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="S30" s="3" t="n">
+      <c r="S30" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T30" s="4" t="inlineStr">
@@ -4574,10 +4576,10 @@
       <c r="V30" s="5" t="n">
         <v>0.004673807205452775</v>
       </c>
-      <c r="W30" s="3" t="n">
+      <c r="W30" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="X30" s="3" t="n">
+      <c r="X30" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y30" s="4" t="inlineStr">
@@ -4591,10 +4593,10 @@
       <c r="AA30" s="5" t="n">
         <v>0.004194756554307116</v>
       </c>
-      <c r="AB30" s="3" t="n">
+      <c r="AB30" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="AC30" s="3" t="n">
+      <c r="AC30" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD30" s="4" t="inlineStr">
@@ -4623,10 +4625,10 @@
           <t>宁夏回族自治区</t>
         </is>
       </c>
-      <c r="C31" s="3" t="n">
+      <c r="C31" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="D31" s="3" t="n">
+      <c r="D31" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -4640,10 +4642,10 @@
       <c r="G31" s="5" t="n">
         <v>0.004454342984409799</v>
       </c>
-      <c r="H31" s="3" t="n">
+      <c r="H31" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="I31" s="3" t="n">
+      <c r="I31" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -4657,10 +4659,10 @@
       <c r="L31" s="5" t="n">
         <v>0.01079011486251305</v>
       </c>
-      <c r="M31" s="3" t="n">
+      <c r="M31" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="N31" s="3" t="n">
+      <c r="N31" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O31" s="4" t="inlineStr">
@@ -4674,10 +4676,10 @@
       <c r="Q31" s="5" t="n">
         <v>0.006058770069675856</v>
       </c>
-      <c r="R31" s="3" t="n">
+      <c r="R31" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="S31" s="3" t="n">
+      <c r="S31" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
@@ -4691,10 +4693,10 @@
       <c r="V31" s="5" t="n">
         <v>0.006523855890944498</v>
       </c>
-      <c r="W31" s="3" t="n">
+      <c r="W31" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="X31" s="3" t="n">
+      <c r="X31" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y31" s="4" t="inlineStr">
@@ -4708,10 +4710,10 @@
       <c r="AA31" s="5" t="n">
         <v>0.007228464419475655</v>
       </c>
-      <c r="AB31" s="3" t="n">
+      <c r="AB31" s="9" t="n">
         <v>46418</v>
       </c>
-      <c r="AC31" s="3" t="n">
+      <c r="AC31" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD31" s="4" t="inlineStr">
@@ -4740,10 +4742,10 @@
           <t>新疆维吾尔自治区</t>
         </is>
       </c>
-      <c r="C32" s="3" t="n">
+      <c r="C32" s="9" t="n">
         <v>46397</v>
       </c>
-      <c r="D32" s="3" t="n">
+      <c r="D32" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -4757,10 +4759,10 @@
       <c r="G32" s="5" t="n">
         <v>0.01187824795842613</v>
       </c>
-      <c r="H32" s="3" t="n">
+      <c r="H32" s="9" t="n">
         <v>46397</v>
       </c>
-      <c r="I32" s="3" t="n">
+      <c r="I32" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -4774,10 +4776,10 @@
       <c r="L32" s="5" t="n">
         <v>0.01949182039679777</v>
       </c>
-      <c r="M32" s="3" t="n">
+      <c r="M32" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="N32" s="3" t="n">
+      <c r="N32" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="O32" s="4" t="inlineStr">
@@ -4791,10 +4793,10 @@
       <c r="Q32" s="5" t="n">
         <v>0.01726749469857619</v>
       </c>
-      <c r="R32" s="3" t="n">
+      <c r="R32" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="S32" s="3" t="n">
+      <c r="S32" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="T32" s="4" t="inlineStr">
@@ -4808,10 +4810,10 @@
       <c r="V32" s="5" t="n">
         <v>0.01772151898734177</v>
       </c>
-      <c r="W32" s="3" t="n">
+      <c r="W32" s="9" t="n">
         <v>46404</v>
       </c>
-      <c r="X32" s="3" t="n">
+      <c r="X32" s="9" t="n">
         <v>46440</v>
       </c>
       <c r="Y32" s="4" t="inlineStr">
@@ -4825,10 +4827,10 @@
       <c r="AA32" s="5" t="n">
         <v>0.01962546816479401</v>
       </c>
-      <c r="AB32" s="3" t="n">
+      <c r="AB32" s="9" t="n">
         <v>46411</v>
       </c>
-      <c r="AC32" s="3" t="n">
+      <c r="AC32" s="9" t="n">
         <v>46433</v>
       </c>
       <c r="AD32" s="4" t="inlineStr">
@@ -5086,6 +5088,129 @@
       <c r="B10" s="8" t="inlineStr">
         <is>
           <t>在“省份日历_人数底表”更新日期或人数后，可通过脚本重跑生成最新版；“来源监控”用于配置官方公告检查来源。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>刷新时间</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>候选数</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>自动更新数</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>保留预估数</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Git同步状态</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-23 11:27:54</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>31</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>刷新时间</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>省份</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>放假日期</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>开学日期</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>置信度</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>来源URL</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>处理结果</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-07-23 11:42:58 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5158,6 +5158,32 @@
         </is>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-23 11:42:57</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>31</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-07-24 05:22:02 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5184,6 +5184,32 @@
         </is>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-24 05:22:01</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>31</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-07-25 05:16:34 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5210,6 +5210,32 @@
         </is>
       </c>
       <c r="F4" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-25 05:16:34</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>31</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-07-26 05:33:55 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5236,6 +5236,32 @@
         </is>
       </c>
       <c r="F5" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-26 05:33:55</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>31</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-07-27 05:52:05 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5262,6 +5262,32 @@
         </is>
       </c>
       <c r="F6" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-27 05:52:05</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>31</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-07-28 05:16:35 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5288,6 +5288,32 @@
         </is>
       </c>
       <c r="F7" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-28 05:16:35</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>31</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-07-29 05:23:46 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5314,6 +5314,32 @@
         </is>
       </c>
       <c r="F8" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-29 05:23:46</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>31</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-07-29 09:22:29 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5340,6 +5340,32 @@
         </is>
       </c>
       <c r="F9" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-29 09:22:27</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>31</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-07-30 05:11:32 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5366,6 +5366,32 @@
         </is>
       </c>
       <c r="F10" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-30 05:11:32</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>31</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-07-31 05:37:48 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5392,6 +5392,32 @@
         </is>
       </c>
       <c r="F11" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-31 05:37:48</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>31</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-01 05:30:16 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5418,6 +5418,32 @@
         </is>
       </c>
       <c r="F12" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-01 05:30:16</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>31</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-02 05:29:58 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5444,6 +5444,32 @@
         </is>
       </c>
       <c r="F13" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-02 05:29:58</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>31</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-03 05:45:01 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5470,6 +5470,32 @@
         </is>
       </c>
       <c r="F14" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-03 05:45:01</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>31</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-04 05:17:03 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5496,6 +5496,32 @@
         </is>
       </c>
       <c r="F15" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-04 05:17:03</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>31</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-05 05:17:09 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5522,6 +5522,32 @@
         </is>
       </c>
       <c r="F16" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-05 05:17:09</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>31</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-06 05:20:13 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5847,7 +5847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6111,6 +6111,32 @@
         </is>
       </c>
       <c r="F10" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-06 05:20:13</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>31</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-07 04:27:52 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5548,6 +5548,32 @@
         </is>
       </c>
       <c r="F17" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:27:52</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>31</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-08 03:27:30 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5574,6 +5574,32 @@
         </is>
       </c>
       <c r="F18" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-08 03:27:29</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>31</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-09 03:45:03 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5600,6 +5600,32 @@
         </is>
       </c>
       <c r="F19" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-09 03:45:03</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>31</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-10 03:58:31 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5626,6 +5626,32 @@
         </is>
       </c>
       <c r="F20" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-10 03:58:30</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>31</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-11 03:46:50 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5102,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5652,6 +5652,32 @@
         </is>
       </c>
       <c r="F21" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-11 03:46:49</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" t="n">
+        <v>31</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-12 04:09:57 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5698,6 +5698,32 @@
         </is>
       </c>
       <c r="F22" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-12 04:09:57</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>31</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-13 04:14:10 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5724,6 +5724,32 @@
         </is>
       </c>
       <c r="F23" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-13 04:14:10</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>31</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-14 04:11:24 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5750,6 +5750,32 @@
         </is>
       </c>
       <c r="F24" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-14 04:11:24</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
+        <v>31</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-15 02:53:29 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5776,6 +5776,32 @@
         </is>
       </c>
       <c r="F25" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-15 02:53:28</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="n">
+        <v>31</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-16 03:02:32 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5802,6 +5802,32 @@
         </is>
       </c>
       <c r="F26" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-16 03:02:31</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>31</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-17 03:01:42 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5828,6 +5828,32 @@
         </is>
       </c>
       <c r="F27" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-17 03:01:41</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
+        <v>31</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-18 02:57:07 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5854,6 +5854,32 @@
         </is>
       </c>
       <c r="F28" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-18 02:57:07</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>31</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-19 02:58:47 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5880,6 +5880,32 @@
         </is>
       </c>
       <c r="F29" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-19 02:58:46</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>31</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-20 02:58:50 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5906,6 +5906,32 @@
         </is>
       </c>
       <c r="F30" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-20 02:58:49</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>31</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-21 03:04:28 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5932,6 +5932,32 @@
         </is>
       </c>
       <c r="F31" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-21 03:04:28</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>31</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-22 02:55:22 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5958,6 +5958,32 @@
         </is>
       </c>
       <c r="F32" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-22 02:55:22</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>31</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-23 03:04:21 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5984,6 +5984,32 @@
         </is>
       </c>
       <c r="F33" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-23 03:04:21</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>31</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-24 03:04:58 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6010,6 +6010,32 @@
         </is>
       </c>
       <c r="F34" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-24 03:04:57</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
+        <v>31</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-25 03:00:44 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6036,6 +6036,32 @@
         </is>
       </c>
       <c r="F35" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-25 03:00:44</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
+        <v>31</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-26 03:06:32 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6062,6 +6062,32 @@
         </is>
       </c>
       <c r="F36" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-26 03:06:31</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>31</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-27 12:26:09 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6088,6 +6088,32 @@
         </is>
       </c>
       <c r="F37" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-27 12:26:08</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>31</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-28 13:54:42 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6114,6 +6114,32 @@
         </is>
       </c>
       <c r="F38" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-28 13:54:41</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="n">
+        <v>31</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-29 08:42:47 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6140,6 +6140,32 @@
         </is>
       </c>
       <c r="F39" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-29 08:42:47</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" t="n">
+        <v>31</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-30 08:00:02 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6166,6 +6166,32 @@
         </is>
       </c>
       <c r="F40" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-30 08:00:02</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" t="n">
+        <v>31</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-08-31 08:14:14 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6192,6 +6192,32 @@
         </is>
       </c>
       <c r="F41" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-08-31 08:14:14</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="n">
+        <v>31</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-01 07:25:01 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6218,6 +6218,32 @@
         </is>
       </c>
       <c r="F42" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-09-01 07:25:00</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="n">
+        <v>31</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-02 06:53:59 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6244,6 +6244,32 @@
         </is>
       </c>
       <c r="F43" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-09-02 06:53:59</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="n">
+        <v>31</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-03 06:57:47 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6270,6 +6270,32 @@
         </is>
       </c>
       <c r="F44" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-09-03 06:57:47</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>31</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-04 07:01:26 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6296,6 +6296,32 @@
         </is>
       </c>
       <c r="F45" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-09-04 07:01:26</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" t="n">
+        <v>31</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-05 06:46:33 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6322,6 +6322,32 @@
         </is>
       </c>
       <c r="F46" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-09-05 06:46:32</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" t="n">
+        <v>31</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-06 06:57:10 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6348,6 +6348,32 @@
         </is>
       </c>
       <c r="F47" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-09-06 06:57:10</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" t="n">
+        <v>31</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-07 07:05:57 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6374,6 +6374,32 @@
         </is>
       </c>
       <c r="F48" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-09-07 07:05:57</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" t="n">
+        <v>31</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-08 07:00:13 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6400,6 +6400,32 @@
         </is>
       </c>
       <c r="F49" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-09-08 07:00:13</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" t="n">
+        <v>31</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-09 07:09:22 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6426,6 +6426,32 @@
         </is>
       </c>
       <c r="F50" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09-09 07:09:22</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" t="n">
+        <v>31</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-10 07:05:58 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6452,6 +6452,32 @@
         </is>
       </c>
       <c r="F51" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-10 07:05:58</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" t="n">
+        <v>31</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-11 07:05:07 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6478,6 +6478,32 @@
         </is>
       </c>
       <c r="F52" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-09-11 07:05:07</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" t="n">
+        <v>31</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-12 06:57:45 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6504,6 +6504,32 @@
         </is>
       </c>
       <c r="F53" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-09-12 06:57:45</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" t="n">
+        <v>31</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-13 07:15:53 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6530,6 +6530,32 @@
         </is>
       </c>
       <c r="F54" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-09-13 07:15:53</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" t="n">
+        <v>31</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>